<commit_message>
Deploying to main from @ pedalboard/pedalboard-hw@b49919d0ec7fda196d9a417ab4be2f565c2a4e34 🚀
</commit_message>
<xml_diff>
--- a/latest/BoM/Generic/pedalboard-hw-bom.xlsx
+++ b/latest/BoM/Generic/pedalboard-hw-bom.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="376">
   <si>
     <t>Row</t>
   </si>
@@ -58,6 +58,9 @@
     <t>Digikey</t>
   </si>
   <si>
+    <t>Sim.Pins</t>
+  </si>
+  <si>
     <t>Mouser</t>
   </si>
   <si>
@@ -250,6 +253,9 @@
     <t>10</t>
   </si>
   <si>
+    <t>Light emitting diode</t>
+  </si>
+  <si>
     <t>LED</t>
   </si>
   <si>
@@ -262,12 +268,15 @@
     <t>LED_0805_2012Metric</t>
   </si>
   <si>
-    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/3739/B1701URO-20D000114U1930.pdf</t>
+    <t>~</t>
   </si>
   <si>
     <t>https://www.digikey.ch/en/products/detail/harvatek-corporation/B1701URO-20D000114U1930/16671739</t>
   </si>
   <si>
+    <t>1=K 2=A</t>
+  </si>
+  <si>
     <t>11</t>
   </si>
   <si>
@@ -277,9 +286,6 @@
     <t>LED Y</t>
   </si>
   <si>
-    <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/docus/3804/B1701NG--20D000314U1930.pdf</t>
-  </si>
-  <si>
     <t>https://www.digikey.ch/en/products/detail/harvatek-corporation/B1701NG-20D000314U1930/16671738</t>
   </si>
   <si>
@@ -424,9 +430,6 @@
     <t>Pedalboard_Soundcard</t>
   </si>
   <si>
-    <t>~</t>
-  </si>
-  <si>
     <t>19</t>
   </si>
   <si>
@@ -550,6 +553,9 @@
     <t>25</t>
   </si>
   <si>
+    <t>Resistor, small symbol</t>
+  </si>
+  <si>
     <t>R_Small</t>
   </si>
   <si>
@@ -562,9 +568,6 @@
     <t>R_0805_2012Metric</t>
   </si>
   <si>
-    <t>https://www.seielect.com/catalog/sei-rncp.pdf</t>
-  </si>
-  <si>
     <t>https://www.digikey.ch/de/products/detail/stackpole-electronics-inc/RNCP0805FTD10R0/2240197</t>
   </si>
   <si>
@@ -580,9 +583,6 @@
     <t>27R</t>
   </si>
   <si>
-    <t>https://www.seielect.com/catalog/sei-rmcf_rmcp.pdf</t>
-  </si>
-  <si>
     <t>https://www.digikey.ch/de/products/detail/stackpole-electronics-inc/RMCF0805FT27R0/1712920</t>
   </si>
   <si>
@@ -1024,7 +1024,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>8.0.6+1</t>
+    <t>9.0.1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -1033,13 +1033,13 @@
     <t>Component Count:</t>
   </si>
   <si>
-    <t>138 (117 SMD/ 20 THT)</t>
+    <t>138 (118 SMD/ 20 THT)</t>
   </si>
   <si>
     <t>Fitted Components:</t>
   </si>
   <si>
-    <t>128 (114 SMD/ 13 THT)</t>
+    <t>128 (115 SMD/ 13 THT)</t>
   </si>
   <si>
     <t>Number of PCBs:</t>
@@ -1067,6 +1067,9 @@
   </si>
   <si>
     <t>https://www.digikey.ch/de/products/detail/w%C3%BCrth-elektronik/694106301002/5047522</t>
+  </si>
+  <si>
+    <t>5-pin DIN connector (5-pin DIN-5 stereo)</t>
   </si>
   <si>
     <t>DIN-5_180degree</t>
@@ -1314,10 +1317,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>2519775</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>297815</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1464384</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>123779</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1344,7 +1347,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9396825" cy="5079365"/>
+          <a:ext cx="2378784" cy="1285829"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1366,10 +1369,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>2157825</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>107315</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1464384</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>123779</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1396,7 +1399,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9396825" cy="5079365"/>
+          <a:ext cx="2378784" cy="1285829"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1693,7 +1696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1708,12 +1711,13 @@
     <col min="10" max="10" width="60.7109375" customWidth="1"/>
     <col min="11" max="11" width="60.7109375" customWidth="1"/>
     <col min="12" max="12" width="19.7109375" customWidth="1"/>
-    <col min="13" max="13" width="19.7109375" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" customWidth="1"/>
-    <col min="15" max="15" width="22.7109375" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" customWidth="1"/>
+    <col min="14" max="14" width="19.7109375" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" customWidth="1"/>
+    <col min="16" max="16" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="32" customHeight="1">
+    <row r="1" spans="1:16" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
         <v>324</v>
       </c>
@@ -1729,8 +1733,9 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
-    </row>
-    <row r="2" spans="1:15">
+      <c r="P1" s="1"/>
+    </row>
+    <row r="2" spans="1:16">
       <c r="C2" s="2" t="s">
         <v>325</v>
       </c>
@@ -1744,7 +1749,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:16">
       <c r="C3" s="2" t="s">
         <v>327</v>
       </c>
@@ -1758,7 +1763,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:16">
       <c r="C4" s="2" t="s">
         <v>329</v>
       </c>
@@ -1772,7 +1777,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:16">
       <c r="C5" s="2" t="s">
         <v>331</v>
       </c>
@@ -1786,7 +1791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:16">
       <c r="C6" s="2" t="s">
         <v>333</v>
       </c>
@@ -1800,7 +1805,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:16">
       <c r="A8" s="4" t="s">
         <v>0</v>
       </c>
@@ -1846,1238 +1851,1319 @@
       <c r="O8" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" ht="30" customHeight="1">
+      <c r="P8" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="30" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="30" customHeight="1">
+      <c r="A10" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M10" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N10" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O10" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P10" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="30" customHeight="1">
+      <c r="A11" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="30" customHeight="1">
+      <c r="A12" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="H12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P12" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="30" customHeight="1">
+      <c r="A13" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="5" t="s">
+      <c r="D13" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="G13" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="30" customHeight="1">
+      <c r="A14" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="H14" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="J9" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="L9" s="6" t="s">
+      <c r="I14" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="K14" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O14" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P14" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="30" customHeight="1">
+      <c r="A15" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P15" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="30" customHeight="1">
+      <c r="A16" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="L16" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M16" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N16" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O16" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P16" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="45" customHeight="1">
+      <c r="A17" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="H17" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O17" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P17" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="30" customHeight="1">
+      <c r="A18" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="G18" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="H18" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M18" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="N18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O18" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P18" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="30" customHeight="1">
+      <c r="A19" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="30" customHeight="1">
+      <c r="A20" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="6" t="s">
+      <c r="H20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="K20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O20" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P20" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="30" customHeight="1">
+      <c r="A21" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" ht="30" customHeight="1">
-      <c r="A10" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="10" t="s">
+      <c r="H21" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P21" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="30" customHeight="1">
+      <c r="A22" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="G22" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H10" s="9" t="s">
+      <c r="H22" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="K22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P22" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="30" customHeight="1">
+      <c r="A23" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O23" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P23" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="30" customHeight="1">
+      <c r="A24" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="G24" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="H24" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="J10" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="K10" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="L10" s="10" t="s">
+      <c r="I24" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="L24" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M24" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N24" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O24" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P24" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="30" customHeight="1">
+      <c r="A25" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P25" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16">
+      <c r="A26" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="G26" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="M10" s="10" t="s">
+      <c r="H26" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="J26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P26" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="30" customHeight="1">
+      <c r="A27" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="N10" s="10" t="s">
+      <c r="H27" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P27" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="30" customHeight="1">
+      <c r="A28" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="G28" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="10" t="s">
+      <c r="H28" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="K28" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L28" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M28" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N28" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O28" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P28" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="30" customHeight="1">
+      <c r="A29" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="G29" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" ht="30" customHeight="1">
-      <c r="A11" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="6" t="s">
+      <c r="H29" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P29" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="30" customHeight="1">
+      <c r="A30" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="K30" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L30" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M30" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N30" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O30" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P30" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="30" customHeight="1">
+      <c r="A31" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="G31" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H11" s="5" t="s">
+      <c r="H31" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P31" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="30" customHeight="1">
+      <c r="A32" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="K32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O32" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P32" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="30" customHeight="1">
+      <c r="A33" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="G33" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="I11" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O11" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" ht="30" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="9" t="s">
+      <c r="H33" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="K33" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N33" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="P33" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="30" customHeight="1">
+      <c r="A34" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="G34" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="I12" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="J12" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="K12" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O12" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" ht="30" customHeight="1">
-      <c r="A13" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="L13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="M13" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O13" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" ht="30" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="J14" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="K14" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M14" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N14" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O14" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="K15" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N15" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O15" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="30" customHeight="1">
-      <c r="A16" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="K16" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="L16" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M16" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N16" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O16" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="45" customHeight="1">
-      <c r="A17" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="K17" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="L17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N17" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O17" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="30" customHeight="1">
-      <c r="A18" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="J18" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="K18" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="L18" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M18" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N18" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O18" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" ht="30" customHeight="1">
-      <c r="A19" s="5" t="s">
+      <c r="H34" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I34" s="10" t="s">
         <v>82</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="J19" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L19" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N19" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O19" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" ht="30" customHeight="1">
-      <c r="A20" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I20" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="J20" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="K20" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="L20" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M20" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N20" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O20" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="30" customHeight="1">
-      <c r="A21" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I21" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O21" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" ht="30" customHeight="1">
-      <c r="A22" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I22" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="J22" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="K22" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="L22" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M22" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N22" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O22" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" ht="30" customHeight="1">
-      <c r="A23" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="J23" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="K23" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L23" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M23" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N23" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O23" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" ht="30" customHeight="1">
-      <c r="A24" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="F24" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H24" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I24" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="J24" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="K24" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="L24" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M24" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N24" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O24" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" ht="30" customHeight="1">
-      <c r="A25" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="K25" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="L25" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M25" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N25" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O25" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15">
-      <c r="A26" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="E26" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="F26" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="G26" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="J26" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="K26" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="L26" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M26" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N26" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O26" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" ht="30" customHeight="1">
-      <c r="A27" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="K27" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L27" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M27" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N27" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O27" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" ht="30" customHeight="1">
-      <c r="A28" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="E28" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="F28" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I28" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="J28" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="K28" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="L28" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M28" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N28" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O28" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" ht="30" customHeight="1">
-      <c r="A29" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="J29" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="K29" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="L29" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M29" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N29" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O29" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" ht="30" customHeight="1">
-      <c r="A30" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H30" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I30" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="J30" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="K30" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="L30" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M30" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N30" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O30" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" ht="30" customHeight="1">
-      <c r="A31" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="J31" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="K31" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="L31" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M31" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N31" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O31" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" ht="30" customHeight="1">
-      <c r="A32" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="D32" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I32" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="J32" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="K32" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="L32" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M32" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N32" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O32" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" ht="30" customHeight="1">
-      <c r="A33" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I33" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="J33" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="K33" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="M33" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="N33" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="O33" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" ht="30" customHeight="1">
-      <c r="A34" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="B34" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>185</v>
-      </c>
-      <c r="F34" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H34" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I34" s="11" t="s">
-        <v>186</v>
       </c>
       <c r="J34" s="12" t="s">
         <v>187</v>
       </c>
       <c r="K34" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L34" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M34" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N34" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O34" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P34" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="30" customHeight="1">
       <c r="A35" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>16</v>
+      <c r="B35" s="8" t="s">
+        <v>177</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>189</v>
@@ -3086,45 +3172,48 @@
         <v>190</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I35" s="7" t="s">
-        <v>186</v>
+        <v>23</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="J35" s="8" t="s">
         <v>191</v>
       </c>
       <c r="K35" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M35" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O35" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P35" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="30" customHeight="1">
       <c r="A36" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="B36" s="10" t="s">
-        <v>16</v>
+      <c r="B36" s="12" t="s">
+        <v>177</v>
       </c>
       <c r="C36" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D36" s="11" t="s">
         <v>193</v>
@@ -3133,45 +3222,48 @@
         <v>194</v>
       </c>
       <c r="F36" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I36" s="11" t="s">
-        <v>186</v>
+        <v>23</v>
+      </c>
+      <c r="I36" s="10" t="s">
+        <v>82</v>
       </c>
       <c r="J36" s="12" t="s">
         <v>195</v>
       </c>
       <c r="K36" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M36" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N36" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O36" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P36" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="30" customHeight="1">
       <c r="A37" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>16</v>
+      <c r="B37" s="8" t="s">
+        <v>177</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>197</v>
@@ -3180,45 +3272,48 @@
         <v>198</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I37" s="7" t="s">
-        <v>180</v>
+        <v>23</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="J37" s="8" t="s">
         <v>199</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M37" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N37" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O37" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P37" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="30" customHeight="1">
       <c r="A38" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B38" s="10" t="s">
-        <v>16</v>
+      <c r="B38" s="12" t="s">
+        <v>177</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D38" s="11" t="s">
         <v>201</v>
@@ -3227,16 +3322,16 @@
         <v>202</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I38" s="11" t="s">
-        <v>180</v>
+        <v>23</v>
+      </c>
+      <c r="I38" s="10" t="s">
+        <v>82</v>
       </c>
       <c r="J38" s="12" t="s">
         <v>203</v>
@@ -3245,27 +3340,30 @@
         <v>204</v>
       </c>
       <c r="L38" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M38" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N38" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O38" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P38" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="30" customHeight="1">
       <c r="A39" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>16</v>
+      <c r="B39" s="8" t="s">
+        <v>177</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D39" s="7" t="s">
         <v>206</v>
@@ -3274,45 +3372,48 @@
         <v>207</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>180</v>
+        <v>23</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="J39" s="8" t="s">
         <v>208</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M39" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N39" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O39" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P39" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="30" customHeight="1">
       <c r="A40" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B40" s="10" t="s">
-        <v>16</v>
+      <c r="B40" s="12" t="s">
+        <v>177</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D40" s="11" t="s">
         <v>210</v>
@@ -3321,16 +3422,16 @@
         <v>211</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I40" s="11" t="s">
-        <v>180</v>
+        <v>23</v>
+      </c>
+      <c r="I40" s="10" t="s">
+        <v>82</v>
       </c>
       <c r="J40" s="12" t="s">
         <v>199</v>
@@ -3339,27 +3440,30 @@
         <v>212</v>
       </c>
       <c r="L40" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M40" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N40" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O40" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P40" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" ht="30" customHeight="1">
       <c r="A41" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>16</v>
+      <c r="B41" s="8" t="s">
+        <v>177</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>214</v>
@@ -3368,16 +3472,16 @@
         <v>215</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I41" s="7" t="s">
-        <v>186</v>
+        <v>23</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="J41" s="8" t="s">
         <v>216</v>
@@ -3386,27 +3490,30 @@
         <v>217</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M41" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N41" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O41" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P41" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="30" customHeight="1">
       <c r="A42" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="B42" s="10" t="s">
-        <v>16</v>
+      <c r="B42" s="12" t="s">
+        <v>177</v>
       </c>
       <c r="C42" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D42" s="11" t="s">
         <v>219</v>
@@ -3415,42 +3522,45 @@
         <v>220</v>
       </c>
       <c r="F42" s="11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I42" s="11" t="s">
-        <v>180</v>
+        <v>23</v>
+      </c>
+      <c r="I42" s="10" t="s">
+        <v>82</v>
       </c>
       <c r="J42" s="12" t="s">
         <v>199</v>
       </c>
       <c r="K42" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L42" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M42" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N42" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O42" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P42" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" ht="30" customHeight="1">
       <c r="A43" s="5" t="s">
         <v>221</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C43" s="7" t="s">
         <v>222</v>
@@ -3465,10 +3575,10 @@
         <v>225</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I43" s="7" t="s">
         <v>226</v>
@@ -3480,24 +3590,27 @@
         <v>228</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O43" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P43" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="30" customHeight="1">
       <c r="A44" s="9" t="s">
         <v>229</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>230</v>
@@ -3512,10 +3625,10 @@
         <v>233</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I44" s="11" t="s">
         <v>234</v>
@@ -3527,24 +3640,27 @@
         <v>236</v>
       </c>
       <c r="L44" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M44" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N44" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O44" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="45" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P44" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="30" customHeight="1">
       <c r="A45" s="5" t="s">
         <v>237</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C45" s="7" t="s">
         <v>238</v>
@@ -3559,10 +3675,10 @@
         <v>240</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I45" s="7" t="s">
         <v>241</v>
@@ -3571,27 +3687,30 @@
         <v>242</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O45" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P45" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="30" customHeight="1">
       <c r="A46" s="9" t="s">
         <v>243</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C46" s="11" t="s">
         <v>244</v>
@@ -3606,10 +3725,10 @@
         <v>246</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I46" s="11" t="s">
         <v>247</v>
@@ -3618,27 +3737,30 @@
         <v>248</v>
       </c>
       <c r="K46" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L46" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M46" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N46" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="N46" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O46" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="O46" s="12" t="s">
+      <c r="P46" s="12" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="47" spans="1:15" ht="45" customHeight="1">
+    <row r="47" spans="1:16" ht="45" customHeight="1">
       <c r="A47" s="5" t="s">
         <v>250</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C47" s="7" t="s">
         <v>251</v>
@@ -3653,10 +3775,10 @@
         <v>254</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I47" s="7" t="s">
         <v>255</v>
@@ -3665,22 +3787,25 @@
         <v>256</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M47" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O47" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P47" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="30" customHeight="1">
       <c r="A48" s="9" t="s">
         <v>257</v>
       </c>
@@ -3700,10 +3825,10 @@
         <v>261</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I48" s="11" t="s">
         <v>262</v>
@@ -3712,22 +3837,25 @@
         <v>263</v>
       </c>
       <c r="K48" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L48" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M48" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N48" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O48" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P48" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" ht="30" customHeight="1">
       <c r="A49" s="5" t="s">
         <v>264</v>
       </c>
@@ -3747,10 +3875,10 @@
         <v>268</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I49" s="7" t="s">
         <v>269</v>
@@ -3759,27 +3887,30 @@
         <v>270</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P49" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" ht="30" customHeight="1">
       <c r="A50" s="9" t="s">
         <v>271</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C50" s="11" t="s">
         <v>272</v>
@@ -3794,10 +3925,10 @@
         <v>274</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I50" s="11" t="s">
         <v>275</v>
@@ -3806,27 +3937,30 @@
         <v>276</v>
       </c>
       <c r="K50" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L50" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M50" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N50" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O50" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P50" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" ht="30" customHeight="1">
       <c r="A51" s="5" t="s">
         <v>277</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>278</v>
@@ -3841,10 +3975,10 @@
         <v>280</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I51" s="7" t="s">
         <v>281</v>
@@ -3853,22 +3987,25 @@
         <v>282</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M51" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O51" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P51" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" ht="30" customHeight="1">
       <c r="A52" s="9" t="s">
         <v>283</v>
       </c>
@@ -3888,10 +4025,10 @@
         <v>287</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I52" s="11" t="s">
         <v>288</v>
@@ -3900,22 +4037,25 @@
         <v>289</v>
       </c>
       <c r="K52" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L52" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M52" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N52" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O52" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P52" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" ht="30" customHeight="1">
       <c r="A53" s="5" t="s">
         <v>290</v>
       </c>
@@ -3935,10 +4075,10 @@
         <v>294</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I53" s="7" t="s">
         <v>295</v>
@@ -3947,22 +4087,25 @@
         <v>296</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M53" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O53" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P53" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" ht="30" customHeight="1">
       <c r="A54" s="9" t="s">
         <v>297</v>
       </c>
@@ -3982,10 +4125,10 @@
         <v>301</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I54" s="11" t="s">
         <v>302</v>
@@ -3994,27 +4137,30 @@
         <v>303</v>
       </c>
       <c r="K54" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L54" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M54" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N54" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O54" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P54" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" ht="30" customHeight="1">
       <c r="A55" s="5" t="s">
         <v>304</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C55" s="7" t="s">
         <v>305</v>
@@ -4029,10 +4175,10 @@
         <v>308</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I55" s="7" t="s">
         <v>309</v>
@@ -4041,27 +4187,30 @@
         <v>310</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O55" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="56" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P55" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="30" customHeight="1">
       <c r="A56" s="9" t="s">
         <v>311</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C56" s="11" t="s">
         <v>312</v>
@@ -4076,10 +4225,10 @@
         <v>314</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I56" s="11" t="s">
         <v>315</v>
@@ -4088,22 +4237,25 @@
         <v>316</v>
       </c>
       <c r="K56" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L56" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M56" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N56" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O56" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P56" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" ht="30" customHeight="1">
       <c r="A57" s="5" t="s">
         <v>317</v>
       </c>
@@ -4123,10 +4275,10 @@
         <v>321</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I57" s="7" t="s">
         <v>322</v>
@@ -4135,24 +4287,27 @@
         <v>323</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O57" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="P57" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C1:O1"/>
+    <mergeCell ref="C1:P1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
@@ -4162,11 +4317,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" customWidth="1"/>
+    <col min="2" max="2" width="45.7109375" customWidth="1"/>
     <col min="3" max="3" width="23.7109375" customWidth="1"/>
     <col min="4" max="4" width="20.7109375" customWidth="1"/>
     <col min="5" max="5" width="28.7109375" customWidth="1"/>
@@ -4177,12 +4332,13 @@
     <col min="10" max="10" width="60.7109375" customWidth="1"/>
     <col min="11" max="11" width="21.7109375" customWidth="1"/>
     <col min="12" max="12" width="17.7109375" customWidth="1"/>
-    <col min="13" max="13" width="16.7109375" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" customWidth="1"/>
     <col min="14" max="14" width="16.7109375" customWidth="1"/>
     <col min="15" max="15" width="16.7109375" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="32" customHeight="1">
+    <row r="1" spans="1:16" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
         <v>324</v>
       </c>
@@ -4198,8 +4354,9 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
-    </row>
-    <row r="2" spans="1:15">
+      <c r="P1" s="1"/>
+    </row>
+    <row r="2" spans="1:16">
       <c r="C2" s="2" t="s">
         <v>325</v>
       </c>
@@ -4213,7 +4370,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:16">
       <c r="C3" s="2" t="s">
         <v>327</v>
       </c>
@@ -4227,7 +4384,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:16">
       <c r="C4" s="2" t="s">
         <v>329</v>
       </c>
@@ -4241,7 +4398,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:16">
       <c r="C5" s="2" t="s">
         <v>331</v>
       </c>
@@ -4255,7 +4412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:16">
       <c r="C6" s="2" t="s">
         <v>333</v>
       </c>
@@ -4269,7 +4426,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:16">
       <c r="A8" s="4" t="s">
         <v>0</v>
       </c>
@@ -4315,13 +4472,16 @@
       <c r="O8" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" ht="30" customHeight="1">
+      <c r="P8" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="30" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>342</v>
@@ -4336,7 +4496,7 @@
         <v>345</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>346</v>
@@ -4348,259 +4508,277 @@
         <v>348</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="30" customHeight="1">
       <c r="A10" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>16</v>
+        <v>22</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>349</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>346</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N10" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O10" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
+        <v>17</v>
+      </c>
+      <c r="P10" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
       <c r="A11" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>346</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>134</v>
+        <v>82</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="30" customHeight="1">
       <c r="A12" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>346</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="O12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="P12" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="A13" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="L12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="N12" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="O12" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
-      <c r="A13" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>362</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>363</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>15</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>346</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>134</v>
+        <v>82</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" ht="30" customHeight="1">
+        <v>17</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="30" customHeight="1">
       <c r="A14" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>230</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>346</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="P14" s="10" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C1:O1"/>
+    <mergeCell ref="C1:P1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
@@ -4618,27 +4796,27 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="7" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="8" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="6" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>